<commit_message>
Update registration center master data
Refreshes the registration center XLSX master datasets, including the main and historical files, to reflect the latest center records and updates.
</commit_message>
<xml_diff>
--- a/mosip_master/xlsx/registration_center.xlsx
+++ b/mosip_master/xlsx/registration_center.xlsx
@@ -55,11 +55,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -546,351 +547,351 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>eng</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>10001</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>SLUDI Suhurupaya Registration Centre</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>REG</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>Suhurupaya Office Complex</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>Subuthipura Road</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>Battaramulla</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>6.9021</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>79.9159</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>0101005-492</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>0112369099</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>Centre Manager</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="M2" s="2" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
+      <c r="N2" s="2" t="inlineStr">
         <is>
           <t>08:00:00</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
+      <c r="O2" s="2" t="inlineStr">
         <is>
           <t>00:10:00</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
+      <c r="P2" s="2" t="inlineStr">
         <is>
           <t>08:00:00</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr">
+      <c r="Q2" s="2" t="inlineStr">
         <is>
           <t>17:00:00</t>
         </is>
       </c>
-      <c r="R2" t="inlineStr">
+      <c r="R2" s="2" t="inlineStr">
         <is>
           <t>12:30:00</t>
         </is>
       </c>
-      <c r="S2" t="inlineStr">
+      <c r="S2" s="2" t="inlineStr">
         <is>
           <t>13:30:00</t>
         </is>
       </c>
-      <c r="T2" t="inlineStr">
+      <c r="T2" s="2" t="inlineStr">
         <is>
           <t>Asia/Colombo</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr">
+      <c r="U2" s="2" t="inlineStr">
         <is>
           <t>LKA</t>
         </is>
       </c>
-      <c r="V2" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="W2" t="inlineStr">
+      <c r="V2" s="2" t="inlineStr">
+        <is>
+          <t>LKA</t>
+        </is>
+      </c>
+      <c r="W2" s="2" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>sin</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>10001</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>SLUDI සුහුරුපාය ලියාපදිංචි මධ්‍යස්ථානය</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>REG</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>සුහුරුපාය කාර්යාල සංකීර්ණය</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>සුභූතිපුර පාර</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>බත්තරමුල්ල</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>6.9021</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>79.9159</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="J3" s="2" t="inlineStr">
         <is>
           <t>0101005-492</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="K3" s="2" t="inlineStr">
         <is>
           <t>0112369099</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="L3" s="2" t="inlineStr">
         <is>
           <t>මධ්‍යස්ථාන කළමනාකරු</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="M3" s="2" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
+      <c r="N3" s="2" t="inlineStr">
         <is>
           <t>08:00:00</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr">
+      <c r="O3" s="2" t="inlineStr">
         <is>
           <t>00:10:00</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr">
+      <c r="P3" s="2" t="inlineStr">
         <is>
           <t>08:00:00</t>
         </is>
       </c>
-      <c r="Q3" t="inlineStr">
+      <c r="Q3" s="2" t="inlineStr">
         <is>
           <t>17:00:00</t>
         </is>
       </c>
-      <c r="R3" t="inlineStr">
+      <c r="R3" s="2" t="inlineStr">
         <is>
           <t>12:30:00</t>
         </is>
       </c>
-      <c r="S3" t="inlineStr">
+      <c r="S3" s="2" t="inlineStr">
         <is>
           <t>13:30:00</t>
         </is>
       </c>
-      <c r="T3" t="inlineStr">
+      <c r="T3" s="2" t="inlineStr">
         <is>
           <t>Asia/Colombo</t>
         </is>
       </c>
-      <c r="U3" t="inlineStr">
+      <c r="U3" s="2" t="inlineStr">
         <is>
           <t>LKA</t>
         </is>
       </c>
-      <c r="V3" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="W3" t="inlineStr">
+      <c r="V3" s="2" t="inlineStr">
+        <is>
+          <t>LKA</t>
+        </is>
+      </c>
+      <c r="W3" s="2" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>tam</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>10001</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>SLUDI சுஹுருபாய பதிவு மையம்</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>REG</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>சுஹுருபாய அலுவலக வளாகம்</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>சுபூதிபுர வீதி</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>பத்தரமுல்லை</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>6.9021</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>79.9159</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="J4" s="2" t="inlineStr">
         <is>
           <t>0101005-492</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="K4" s="2" t="inlineStr">
         <is>
           <t>0112369099</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="L4" s="2" t="inlineStr">
         <is>
           <t>மைய மேலாளர்</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="M4" s="2" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
+      <c r="N4" s="2" t="inlineStr">
         <is>
           <t>08:00:00</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr">
+      <c r="O4" s="2" t="inlineStr">
         <is>
           <t>00:10:00</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr">
+      <c r="P4" s="2" t="inlineStr">
         <is>
           <t>08:00:00</t>
         </is>
       </c>
-      <c r="Q4" t="inlineStr">
+      <c r="Q4" s="2" t="inlineStr">
         <is>
           <t>17:00:00</t>
         </is>
       </c>
-      <c r="R4" t="inlineStr">
+      <c r="R4" s="2" t="inlineStr">
         <is>
           <t>12:30:00</t>
         </is>
       </c>
-      <c r="S4" t="inlineStr">
+      <c r="S4" s="2" t="inlineStr">
         <is>
           <t>13:30:00</t>
         </is>
       </c>
-      <c r="T4" t="inlineStr">
+      <c r="T4" s="2" t="inlineStr">
         <is>
           <t>Asia/Colombo</t>
         </is>
       </c>
-      <c r="U4" t="inlineStr">
+      <c r="U4" s="2" t="inlineStr">
         <is>
           <t>LKA</t>
         </is>
       </c>
-      <c r="V4" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="W4" t="inlineStr">
+      <c r="V4" s="2" t="inlineStr">
+        <is>
+          <t>LKA</t>
+        </is>
+      </c>
+      <c r="W4" s="2" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>

</xml_diff>